<commit_message>
Approved for Biomax Request 1
</commit_message>
<xml_diff>
--- a/LeaveDeduct.xlsx
+++ b/LeaveDeduct.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>EmpId</t>
   </si>
@@ -35,69 +35,12 @@
   <si>
     <t>Salary to be deducted (In days)</t>
   </si>
-  <si>
-    <t>A-22332</t>
-  </si>
-  <si>
-    <t>VIJAY ANAND KAMBLE</t>
-  </si>
-  <si>
-    <t>09:25:50</t>
-  </si>
-  <si>
-    <t>17:23:21</t>
-  </si>
-  <si>
-    <t>478</t>
-  </si>
-  <si>
-    <t>0.5</t>
-  </si>
-  <si>
-    <t>A-23352</t>
-  </si>
-  <si>
-    <t>Abhilash Babu Suryawanshi</t>
-  </si>
-  <si>
-    <t>13:05:43</t>
-  </si>
-  <si>
-    <t>00:00</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>A-240246</t>
-  </si>
-  <si>
-    <t>Shiwani Dilip Turukmane</t>
-  </si>
-  <si>
-    <t>10:30:08</t>
-  </si>
-  <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>A-23353</t>
-  </si>
-  <si>
-    <t>Vijay Kundlik Lambture</t>
-  </si>
-  <si>
-    <t>12:38:38</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="dd-MM-yyyy"/>
-    <numFmt numFmtId="166" formatCode="dd-MM-yyyy HH:mm:ss"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <sz val="11.00"/>
@@ -125,10 +68,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <dxfs count="0"/>
 </styleSheet>
@@ -142,10 +83,10 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="23.42578125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="8.42578125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="9.42578125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="6.42578125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="9.42578125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="5.42578125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="8.42578125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="9.42578125" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="20.42578125" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="32.42578125" customWidth="true" bestFit="true"/>
@@ -174,29 +115,6 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>45721.0</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="0" useFirstPageNumber="false" blackAndWhite="false" orientation="portrait"/>

</xml_diff>